<commit_message>
upload data tambahan 3500 PO
</commit_message>
<xml_diff>
--- a/salin/List_po_3520.XLSX
+++ b/salin/List_po_3520.XLSX
@@ -6337,10 +6337,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -6384,7 +6389,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -6396,6 +6401,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6677,7 +6688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J1756"/>
+  <dimension ref="A1:N1756"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -6690,8 +6701,8 @@
     <col min="9" max="10" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:14" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
         <v>2094</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -6706,7 +6717,7 @@
       <c r="E1" s="1" t="s">
         <v>2097</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="5" t="s">
         <v>2098</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -6722,7 +6733,7 @@
         <v>2102</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -6754,7 +6765,7 @@
         <v>56011770</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -6786,7 +6797,7 @@
         <v>33800000</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -6818,7 +6829,7 @@
         <v>15116220</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -6850,7 +6861,7 @@
         <v>3234960</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -6882,7 +6893,7 @@
         <v>1076600</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -6914,7 +6925,7 @@
         <v>3640872</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -6946,7 +6957,7 @@
         <v>7835000</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -6977,8 +6988,9 @@
       <c r="J9" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="N9" s="4"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -7010,7 +7022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -7042,7 +7054,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -7074,7 +7086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -7106,7 +7118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -7138,7 +7150,7 @@
         <v>22003000</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -7170,7 +7182,7 @@
         <v>350000</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>33</v>
       </c>
@@ -62883,9 +62895,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1756"/>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>